<commit_message>
feat(vba): Support 4 row header format and targeted caching
- Updated Row trigger boundary to Row 5
- Updated Enum Key read target to Row 3
- Added GetRequiredEnumKeys to pre-scan Data sheets for used Keys
- Optimized ScanReferenceFile to only cache explicitly required Enum Keys
- Updated README.md
- Archived support-four-header-rows OpenSpec change
</commit_message>
<xml_diff>
--- a/reference/Form/Test_Contacts.xlsx
+++ b/reference/Form/Test_Contacts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_開發資料\煉丹\表格\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\ExcelEnumSelectionTool\reference\Form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289B0029-C097-4458-8399-6394A0E0D389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D24E4C9-C47A-4798-A2DD-E8D38FF834C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ContactNode" sheetId="1" r:id="rId1"/>
@@ -248,7 +248,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H8" authorId="0" shapeId="0" xr:uid="{02535DC8-D360-4CD6-84CA-8A02019E5726}">
+    <comment ref="H9" authorId="0" shapeId="0" xr:uid="{02535DC8-D360-4CD6-84CA-8A02019E5726}">
       <text>
         <r>
           <rPr>
@@ -290,7 +290,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="176">
   <si>
     <t>素不相識</t>
   </si>
@@ -977,6 +977,14 @@
   </si>
   <si>
     <t>顧客／預設值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MissonType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PassiveAbilityTarget</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1157,7 +1165,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1441,19 +1449,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="H11:H14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="11" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H14" t="s">
         <v>25</v>
       </c>
@@ -1466,34 +1474,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD06145D-4CC0-4C33-8A6D-3EDFE2464C9A}">
-  <dimension ref="A1:W21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:W22"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.375" customWidth="1"/>
-    <col min="3" max="3" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.375" customWidth="1"/>
-    <col min="5" max="5" width="13.625" customWidth="1"/>
-    <col min="6" max="6" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.25" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28.25" customWidth="1"/>
-    <col min="10" max="10" width="25.125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.25" customWidth="1"/>
-    <col min="12" max="12" width="22.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.75" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.28515625" customWidth="1"/>
+    <col min="10" max="10" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.28515625" customWidth="1"/>
+    <col min="12" max="12" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="23" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="30" customWidth="1"/>
-    <col min="16" max="16" width="28.625" customWidth="1"/>
-    <col min="17" max="18" width="24.75" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="21.625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="28.625" customWidth="1"/>
-    <col min="21" max="21" width="24.75" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.75" customWidth="1"/>
-    <col min="23" max="23" width="21.625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="28.5703125" customWidth="1"/>
+    <col min="17" max="18" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="28.5703125" customWidth="1"/>
+    <col min="21" max="21" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="24.7109375" customWidth="1"/>
+    <col min="23" max="23" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>27</v>
       </c>
@@ -1564,7 +1572,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>35</v>
       </c>
@@ -1635,253 +1643,227 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>5</v>
-      </c>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
       <c r="G3" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="10" t="s">
-        <v>5</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="10"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="M3" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="N3" s="8" t="s">
-        <v>5</v>
-      </c>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
       <c r="O3" s="3"/>
       <c r="P3" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="C4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="G4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="T3" s="6" t="s">
+      <c r="H4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="U3" s="6" t="s">
+      <c r="I4" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="V3" s="6" t="s">
+      <c r="K4" s="3"/>
+      <c r="L4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="6" t="s">
+      <c r="M4" s="8" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="N4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="O4" s="3"/>
+      <c r="P4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="R4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="V4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="W4" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>5110101</v>
       </c>
-      <c r="B4" s="1">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1" t="s">
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1" t="s">
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="1">
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="1">
         <v>5201101</v>
       </c>
-      <c r="M4" s="1">
+      <c r="M5" s="1">
         <v>5201102</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N5" s="1">
         <v>5201103</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="O5" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="P5" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="R4" s="1"/>
-      <c r="S4" s="1" t="s">
+      <c r="R5" s="1"/>
+      <c r="S5" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="T4" s="1" t="s">
+      <c r="T5" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="U4" s="1"/>
-      <c r="V4" s="1"/>
-      <c r="W4" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>5110201</v>
-      </c>
-      <c r="B5" s="1">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="1">
-        <v>2</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="J5" s="1">
-        <v>5202101</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="L5" s="1">
-        <v>5204101</v>
-      </c>
-      <c r="M5" s="1">
-        <v>5204102</v>
-      </c>
-      <c r="N5" s="1">
-        <v>5204103</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>91</v>
-      </c>
+      <c r="U5" s="1"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>5120101</v>
+        <v>5110201</v>
       </c>
       <c r="B6" s="1">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
       <c r="G6" s="1" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="7"/>
+        <v>96</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J6" s="1">
+        <v>5202101</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>121</v>
+      </c>
       <c r="L6" s="1">
-        <v>5201103</v>
+        <v>5204101</v>
       </c>
       <c r="M6" s="1">
-        <v>5201104</v>
+        <v>5204102</v>
       </c>
       <c r="N6" s="1">
-        <v>5201105</v>
+        <v>5204103</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>71</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="1" t="s">
-        <v>68</v>
-      </c>
+      <c r="S6" s="1"/>
       <c r="T6" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="U6" s="1"/>
+        <v>86</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>91</v>
+      </c>
       <c r="V6" s="1"/>
       <c r="W6" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>5120102</v>
+        <v>5120101</v>
       </c>
       <c r="B7" s="1">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1895,12 +1877,8 @@
         <v>97</v>
       </c>
       <c r="I7" s="1"/>
-      <c r="J7" s="1">
-        <v>5205101</v>
-      </c>
-      <c r="K7" s="7" t="s">
-        <v>160</v>
-      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="7"/>
       <c r="L7" s="1">
         <v>5201103</v>
       </c>
@@ -1932,165 +1910,161 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>5120301</v>
+        <v>5120102</v>
       </c>
       <c r="B8" s="1">
         <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="1" t="s">
-        <v>50</v>
-      </c>
+      <c r="E8" s="1"/>
       <c r="F8" s="1">
         <v>1</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="J8" s="1"/>
-      <c r="K8" s="7"/>
+        <v>97</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1">
+        <v>5205101</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>160</v>
+      </c>
       <c r="L8" s="1">
-        <v>5203201</v>
+        <v>5201103</v>
       </c>
       <c r="M8" s="1">
-        <v>5203202</v>
+        <v>5201104</v>
       </c>
       <c r="N8" s="1">
-        <v>5203203</v>
+        <v>5201105</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q8" s="1"/>
+        <v>66</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="R8" s="1"/>
-      <c r="S8" s="1"/>
+      <c r="S8" s="1" t="s">
+        <v>68</v>
+      </c>
       <c r="T8" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="U8" s="1"/>
       <c r="V8" s="1"/>
       <c r="W8" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>5120401</v>
+        <v>5120301</v>
       </c>
       <c r="B9" s="1">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F9" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="7"/>
       <c r="L9" s="1">
+        <v>5203201</v>
+      </c>
+      <c r="M9" s="1">
+        <v>5203202</v>
+      </c>
+      <c r="N9" s="1">
+        <v>5203203</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="P9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="V9" s="1"/>
+      <c r="W9" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>5120401</v>
+      </c>
+      <c r="B10" s="1">
+        <v>2</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="1">
+        <v>3</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="J10" s="1"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="1">
         <v>5201201</v>
       </c>
-      <c r="M9" s="1">
+      <c r="M10" s="1">
         <v>5201202</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N10" s="1">
         <v>5201203</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O10" s="7" t="s">
         <v>137</v>
-      </c>
-      <c r="P9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q9" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="W9" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>5130101</v>
-      </c>
-      <c r="B10" s="1">
-        <v>3</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1">
-        <v>1</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1">
-        <v>5205101</v>
-      </c>
-      <c r="K10" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="L10" s="1">
-        <v>5201104</v>
-      </c>
-      <c r="M10" s="1">
-        <v>5201105</v>
-      </c>
-      <c r="N10" s="1">
-        <v>5201106</v>
-      </c>
-      <c r="O10" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="P10" s="1" t="s">
         <v>66</v>
@@ -2100,31 +2074,33 @@
       </c>
       <c r="R10" s="1"/>
       <c r="S10" s="1" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="U10" s="1"/>
-      <c r="V10" s="1"/>
+        <v>79</v>
+      </c>
+      <c r="U10" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>85</v>
+      </c>
       <c r="W10" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>5140101</v>
+        <v>5130101</v>
       </c>
       <c r="B11" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D11" s="1"/>
-      <c r="E11" s="1" t="s">
-        <v>51</v>
-      </c>
+      <c r="E11" s="1"/>
       <c r="F11" s="1">
         <v>1</v>
       </c>
@@ -2135,19 +2111,23 @@
         <v>97</v>
       </c>
       <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="7"/>
+      <c r="J11" s="1">
+        <v>5205101</v>
+      </c>
+      <c r="K11" s="7" t="s">
+        <v>160</v>
+      </c>
       <c r="L11" s="1">
+        <v>5201104</v>
+      </c>
+      <c r="M11" s="1">
+        <v>5201105</v>
+      </c>
+      <c r="N11" s="1">
         <v>5201106</v>
       </c>
-      <c r="M11" s="1">
-        <v>5201107</v>
-      </c>
-      <c r="N11" s="1">
-        <v>5201108</v>
-      </c>
       <c r="O11" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P11" s="1" t="s">
         <v>66</v>
@@ -2165,40 +2145,97 @@
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>5140101</v>
+      </c>
+      <c r="B12" s="1">
+        <v>4</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="1">
+        <v>5201106</v>
+      </c>
+      <c r="M12" s="1">
+        <v>5201107</v>
+      </c>
+      <c r="N12" s="1">
+        <v>5201108</v>
+      </c>
+      <c r="O12" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="R12" s="1"/>
+      <c r="S12" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="T12" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="U12" s="1"/>
+      <c r="V12" s="1"/>
+      <c r="W12" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2209,23 +2246,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED798693-69A8-4E87-ACDD-D72152D78692}">
-  <dimension ref="A1:M15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M16"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.125" customWidth="1"/>
-    <col min="5" max="6" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" customWidth="1"/>
+    <col min="5" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.75" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="15.875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="27.25" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>166</v>
       </c>
@@ -2266,7 +2303,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>167</v>
       </c>
@@ -2305,119 +2342,99 @@
       </c>
       <c r="M2" s="3"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M3" s="3"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>1</v>
-      </c>
-      <c r="B4" s="11">
-        <v>1</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="M4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>1</v>
+      </c>
+      <c r="B5" s="11">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="4" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>2</v>
-      </c>
-      <c r="B5" s="11">
-        <v>1</v>
-      </c>
-      <c r="C5" s="1">
-        <v>2</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
+      <c r="E5" s="1"/>
       <c r="F5" s="1">
         <v>1</v>
       </c>
-      <c r="G5" s="1">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1">
-        <v>1</v>
-      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
-      <c r="L5" s="1">
-        <v>1</v>
-      </c>
+      <c r="L5" s="1"/>
       <c r="M5" s="4" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="11">
         <v>1</v>
       </c>
       <c r="C6" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="1">
         <v>1</v>
@@ -2428,16 +2445,12 @@
       <c r="G6" s="1">
         <v>1</v>
       </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1">
-        <v>1</v>
-      </c>
-      <c r="J6" s="1">
-        <v>1</v>
-      </c>
-      <c r="K6" s="1">
-        <v>1</v>
-      </c>
+      <c r="H6" s="1">
+        <v>1</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
       <c r="L6" s="1">
         <v>1</v>
       </c>
@@ -2445,18 +2458,18 @@
         <v>172</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="11">
         <v>1</v>
       </c>
       <c r="C7" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E7" s="1">
         <v>1</v>
@@ -2468,7 +2481,9 @@
         <v>1</v>
       </c>
       <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
+      <c r="I7" s="1">
+        <v>1</v>
+      </c>
       <c r="J7" s="1">
         <v>1</v>
       </c>
@@ -2482,84 +2497,86 @@
         <v>172</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
+        <v>4</v>
+      </c>
+      <c r="B8" s="11">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1">
+        <v>4</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1">
+        <v>1</v>
+      </c>
+      <c r="K8" s="1">
+        <v>1</v>
+      </c>
+      <c r="L8" s="1">
+        <v>1</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
         <v>5</v>
-      </c>
-      <c r="B8" s="12">
-        <v>2</v>
-      </c>
-      <c r="C8" s="1">
-        <v>1</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1">
-        <v>1</v>
-      </c>
-      <c r="G8" s="13">
-        <v>1</v>
-      </c>
-      <c r="H8" s="13">
-        <v>1</v>
-      </c>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="4" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>6</v>
       </c>
       <c r="B9" s="12">
         <v>2</v>
       </c>
       <c r="C9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E9" s="1"/>
       <c r="F9" s="1">
         <v>1</v>
       </c>
-      <c r="G9" s="1">
-        <v>1</v>
-      </c>
-      <c r="H9" s="1">
+      <c r="G9" s="13">
+        <v>1</v>
+      </c>
+      <c r="H9" s="13">
         <v>1</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
-      <c r="L9" s="1">
-        <v>1</v>
-      </c>
+      <c r="L9" s="1"/>
       <c r="M9" s="4" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B10" s="12">
         <v>2</v>
       </c>
       <c r="C10" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="1">
         <v>1</v>
@@ -2570,16 +2587,12 @@
       <c r="G10" s="1">
         <v>1</v>
       </c>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1">
-        <v>1</v>
-      </c>
-      <c r="J10" s="1">
-        <v>1</v>
-      </c>
-      <c r="K10" s="1">
-        <v>1</v>
-      </c>
+      <c r="H10" s="1">
+        <v>1</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
       <c r="L10" s="1">
         <v>1</v>
       </c>
@@ -2587,18 +2600,18 @@
         <v>170</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B11" s="12">
         <v>2</v>
       </c>
       <c r="C11" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E11" s="1">
         <v>1</v>
@@ -2610,7 +2623,9 @@
         <v>1</v>
       </c>
       <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+      <c r="I11" s="1">
+        <v>1</v>
+      </c>
       <c r="J11" s="1">
         <v>1</v>
       </c>
@@ -2624,86 +2639,88 @@
         <v>170</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
+        <v>8</v>
+      </c>
+      <c r="B12" s="12">
+        <v>2</v>
+      </c>
+      <c r="C12" s="1">
+        <v>4</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="1">
+        <v>1</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1">
+        <v>1</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1</v>
+      </c>
+      <c r="L12" s="1">
+        <v>1</v>
+      </c>
+      <c r="M12" s="4" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
         <v>9</v>
-      </c>
-      <c r="B12" s="11">
-        <v>3</v>
-      </c>
-      <c r="C12" s="1">
-        <v>1</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="13">
-        <v>1</v>
-      </c>
-      <c r="F12" s="1">
-        <v>1</v>
-      </c>
-      <c r="G12" s="1"/>
-      <c r="H12" s="13">
-        <v>1</v>
-      </c>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="13">
-        <v>1</v>
-      </c>
-      <c r="M12" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
-        <v>10</v>
       </c>
       <c r="B13" s="11">
         <v>3</v>
       </c>
       <c r="C13" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="E13" s="13">
         <v>1</v>
       </c>
       <c r="F13" s="1">
         <v>1</v>
       </c>
-      <c r="G13" s="1">
-        <v>1</v>
-      </c>
-      <c r="H13" s="1">
+      <c r="G13" s="1"/>
+      <c r="H13" s="13">
         <v>1</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
-      <c r="L13" s="1">
+      <c r="L13" s="13">
         <v>1</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="11">
         <v>3</v>
       </c>
       <c r="C14" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="1">
         <v>1</v>
@@ -2714,16 +2731,12 @@
       <c r="G14" s="1">
         <v>1</v>
       </c>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1">
-        <v>1</v>
-      </c>
-      <c r="J14" s="1">
-        <v>1</v>
-      </c>
-      <c r="K14" s="1">
-        <v>1</v>
-      </c>
+      <c r="H14" s="1">
+        <v>1</v>
+      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
       <c r="L14" s="1">
         <v>1</v>
       </c>
@@ -2731,40 +2744,79 @@
         <v>171</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="11">
         <v>3</v>
       </c>
       <c r="C15" s="1">
+        <v>3</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+      <c r="F15" s="1">
+        <v>1</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1</v>
+      </c>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1">
+        <v>1</v>
+      </c>
+      <c r="J15" s="1">
+        <v>1</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1">
+        <v>1</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>12</v>
+      </c>
+      <c r="B16" s="11">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1">
         <v>4</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="1">
-        <v>1</v>
-      </c>
-      <c r="F15" s="1">
-        <v>1</v>
-      </c>
-      <c r="G15" s="1">
-        <v>1</v>
-      </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1">
-        <v>1</v>
-      </c>
-      <c r="K15" s="1">
-        <v>1</v>
-      </c>
-      <c r="L15" s="1">
-        <v>1</v>
-      </c>
-      <c r="M15" s="4" t="s">
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1</v>
+      </c>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1">
+        <v>1</v>
+      </c>
+      <c r="K16" s="1">
+        <v>1</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1</v>
+      </c>
+      <c r="M16" s="4" t="s">
         <v>171</v>
       </c>
     </row>
@@ -2776,18 +2828,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08C6B74D-3759-4DEE-BEDB-ADEF3A2F8D1A}">
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.25" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.25" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>95</v>
       </c>
@@ -2807,7 +2859,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>110</v>
       </c>
@@ -2827,47 +2879,41 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <v>5201101</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1">
-        <v>3</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
-        <v>5201102</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>123</v>
@@ -2877,15 +2923,15 @@
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>5201103</v>
+        <v>5201102</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>123</v>
@@ -2895,15 +2941,15 @@
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>5201104</v>
+        <v>5201103</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>123</v>
@@ -2913,15 +2959,15 @@
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>5201105</v>
+        <v>5201104</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>123</v>
@@ -2931,15 +2977,15 @@
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>5201106</v>
+        <v>5201105</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>123</v>
@@ -2949,15 +2995,15 @@
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>5201107</v>
+        <v>5201106</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>123</v>
@@ -2967,15 +3013,15 @@
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>5201108</v>
+        <v>5201107</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>123</v>
@@ -2985,33 +3031,33 @@
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>5201201</v>
+        <v>5201108</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>5201202</v>
+        <v>5201201</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>123</v>
@@ -3021,15 +3067,15 @@
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>5201203</v>
+        <v>5201202</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>123</v>
@@ -3039,33 +3085,33 @@
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>5202101</v>
+        <v>5201203</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>5202102</v>
+        <v>5202101</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>122</v>
@@ -3075,15 +3121,15 @@
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>5202103</v>
+        <v>5202102</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>122</v>
@@ -3093,33 +3139,33 @@
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>5203201</v>
+        <v>5202103</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>5203202</v>
+        <v>5203201</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>124</v>
@@ -3129,15 +3175,15 @@
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>5203203</v>
+        <v>5203202</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>124</v>
@@ -3147,32 +3193,33 @@
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1">
+        <v>4</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>5203203</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1">
         <v>5</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="1">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
         <v>5204101</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E21" s="1">
-        <v>-300</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
-        <v>5204102</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>153</v>
@@ -3181,15 +3228,15 @@
         <v>111</v>
       </c>
       <c r="E22" s="1">
-        <v>-400</v>
+        <v>-300</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>5204103</v>
+        <v>5204102</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>153</v>
@@ -3198,26 +3245,43 @@
         <v>111</v>
       </c>
       <c r="E23" s="1">
-        <v>-500</v>
+        <v>-400</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>5205101</v>
+        <v>5204103</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>111</v>
       </c>
       <c r="E24" s="1">
+        <v>-500</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>5205101</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E25" s="1">
         <v>500</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="F25" s="1" t="s">
         <v>161</v>
       </c>
     </row>

</xml_diff>